<commit_message>
fix WeeklyReportGenerator to adjust freeze pane settings and clear cell values; add ManualReportGenerationTest for report generation validation
</commit_message>
<xml_diff>
--- a/data/divisions.xlsx
+++ b/data/divisions.xlsx
@@ -700,7 +700,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F3" s="6" t="n">
@@ -772,7 +772,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F5" s="6" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
@@ -878,7 +878,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F13" s="6" t="n">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F16" s="6" t="n">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F17" s="6" t="n">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F18" s="6" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F19" s="6" t="n">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F20" s="6" t="n">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F21" s="6" t="n">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F22" s="6" t="n">
@@ -1394,7 +1394,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F23" s="6" t="n">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F28" s="6" t="n">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F29" s="6" t="n">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F30" s="6" t="n">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F33" s="6" t="n">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F38" s="6" t="n">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F39" s="6" t="n">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F41" s="6" t="n">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F45" s="6" t="n">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F47" s="6" t="n">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F52" s="6" t="n">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F53" s="6" t="n">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F58" s="6" t="n">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F59" s="6" t="n">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F62" s="6" t="n">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F63" s="6" t="n">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F64" s="6" t="n">
@@ -2900,7 +2900,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F67" s="6" t="n">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F77" s="6" t="n">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F79" s="6" t="n">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F81" s="6" t="n">
@@ -3486,7 +3486,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F84" s="6" t="n">
@@ -3520,7 +3520,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F85" s="6" t="n">
@@ -3556,7 +3556,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F86" s="6" t="n">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F88" s="6" t="n">
@@ -3658,7 +3658,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F89" s="6" t="n">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F92" s="6" t="n">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F100" s="6" t="n">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F121" s="6" t="n">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F122" s="6" t="n">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F124" s="6" t="n">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F125" s="6" t="n">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F126" s="6" t="n">
@@ -4956,7 +4956,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F127" s="6" t="n">
@@ -5160,7 +5160,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F133" s="6" t="n">
@@ -5194,7 +5194,7 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F134" s="6" t="n">
@@ -5228,7 +5228,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F135" s="6" t="n">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F136" s="6" t="n">
@@ -5296,7 +5296,7 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F137" s="6" t="n">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F138" s="6" t="n">
@@ -5364,7 +5364,7 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F139" s="6" t="n">
@@ -5398,7 +5398,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F140" s="6" t="n">
@@ -5500,7 +5500,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F143" s="6" t="n">
@@ -5568,7 +5568,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F145" s="6" t="n">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F146" s="6" t="n">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F147" s="6" t="n">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F149" s="6" t="n">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F150" s="6" t="n">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F151" s="6" t="n">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F152" s="6" t="n">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F153" s="6" t="n">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F154" s="6" t="n">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F155" s="6" t="n">
@@ -5940,7 +5940,7 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F156" s="6" t="n">
@@ -5972,7 +5972,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F157" s="6" t="n">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F158" s="6" t="n">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F161" s="6" t="n">
@@ -6144,7 +6144,7 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F162" s="6" t="n">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F163" s="6" t="n">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F164" s="6" t="n">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F165" s="6" t="n">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F168" s="6" t="n">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F173" s="6" t="n">
@@ -6558,7 +6558,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F174" s="6" t="n">
@@ -6592,7 +6592,7 @@
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F175" s="6" t="n">
@@ -6662,7 +6662,7 @@
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F177" s="6" t="n">
@@ -6730,7 +6730,7 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F179" s="6" t="n">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F181" s="6" t="n">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F187" s="6" t="n">
@@ -7036,7 +7036,7 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F188" s="6" t="n">
@@ -7072,7 +7072,7 @@
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F189" s="6" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F190" s="6" t="n">
@@ -7350,7 +7350,7 @@
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F197" s="6" t="n">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F199" s="6" t="n">
@@ -7456,7 +7456,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F200" s="6" t="n">
@@ -7488,7 +7488,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F201" s="6" t="n">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F202" s="6" t="n">
@@ -7624,7 +7624,7 @@
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F205" s="6" t="n">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F208" s="6" t="n">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F212" s="6" t="n">
@@ -7896,7 +7896,7 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F213" s="6" t="n">
@@ -7966,7 +7966,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F215" s="6" t="n">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F226" s="6" t="n">
@@ -8826,7 +8826,7 @@
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F240" s="6" t="n">
@@ -9436,7 +9436,7 @@
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F258" s="6" t="n">
@@ -10324,7 +10324,7 @@
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F284" s="6" t="n">
@@ -11354,7 +11354,7 @@
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F314" s="6" t="n">
@@ -11632,7 +11632,7 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F322" s="6" t="n">
@@ -12008,7 +12008,7 @@
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F333" s="6" t="n">
@@ -12142,7 +12142,7 @@
       </c>
       <c r="E337" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F337" s="6" t="n">
@@ -12450,7 +12450,7 @@
       </c>
       <c r="E346" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F346" s="6" t="n">
@@ -12658,7 +12658,7 @@
       </c>
       <c r="E352" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F352" s="6" t="n">
@@ -12692,7 +12692,7 @@
       </c>
       <c r="E353" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F353" s="6" t="n">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="E363" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F363" s="6" t="n">
@@ -13108,7 +13108,7 @@
       </c>
       <c r="E365" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F365" s="6" t="n">
@@ -13176,7 +13176,7 @@
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F367" s="6" t="n">
@@ -13454,7 +13454,7 @@
       </c>
       <c r="E375" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F375" s="6" t="n">
@@ -13624,7 +13624,7 @@
       </c>
       <c r="E380" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F380" s="6" t="n">
@@ -13658,7 +13658,7 @@
       </c>
       <c r="E381" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F381" s="6" t="n">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="E382" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F382" s="6" t="n">
@@ -13726,7 +13726,7 @@
       </c>
       <c r="E383" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F383" s="6" t="n">
@@ -13760,7 +13760,7 @@
       </c>
       <c r="E384" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F384" s="6" t="n">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="E385" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F385" s="6" t="n">
@@ -13828,7 +13828,7 @@
       </c>
       <c r="E386" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F386" s="6" t="n">
@@ -13896,7 +13896,7 @@
       </c>
       <c r="E388" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F388" s="6" t="n">
@@ -14032,7 +14032,7 @@
       </c>
       <c r="E392" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F392" s="6" t="n">
@@ -14538,7 +14538,7 @@
       </c>
       <c r="E407" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F407" s="6" t="n">
@@ -14572,7 +14572,7 @@
       </c>
       <c r="E408" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F408" s="6" t="n">
@@ -15226,7 +15226,7 @@
       </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F427" s="6" t="n">
@@ -15330,7 +15330,7 @@
       </c>
       <c r="E430" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F430" s="6" t="n">
@@ -16082,7 +16082,7 @@
       </c>
       <c r="E452" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F452" s="6" t="n">
@@ -16490,7 +16490,7 @@
       </c>
       <c r="E464" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F464" s="6" t="n">
@@ -16558,7 +16558,7 @@
       </c>
       <c r="E466" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F466" s="6" t="n">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="E467" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F467" s="6" t="n">
@@ -16728,7 +16728,7 @@
       </c>
       <c r="E471" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F471" s="6" t="n">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="E475" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F475" s="6" t="n">
@@ -16974,7 +16974,7 @@
       </c>
       <c r="E478" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F478" s="6" t="n">
@@ -17178,7 +17178,7 @@
       </c>
       <c r="E484" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F484" s="6" t="n">
@@ -17278,7 +17278,7 @@
       </c>
       <c r="E487" s="2" t="inlineStr">
         <is>
-          <t>Асылхановна Аэлита</t>
+          <t>Алимова Аэлита</t>
         </is>
       </c>
       <c r="F487" s="6" t="n">
@@ -17838,7 +17838,7 @@
       </c>
       <c r="E504" s="2" t="inlineStr">
         <is>
-          <t>Байдулаевна Анна</t>
+          <t>Байдаулетова Анна</t>
         </is>
       </c>
       <c r="F504" s="6" t="n">

</xml_diff>